<commit_message>
Adiciona prints de evidências e atualiza planilhas de Casos de testes e Bug report
</commit_message>
<xml_diff>
--- a/docs/Casos de teste - Cadastro de usuário Ecommerce.xlsx
+++ b/docs/Casos de teste - Cadastro de usuário Ecommerce.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\LP7037\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\LP7037\Desktop\projeto qa cadastro de usuario\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F9C9B961-6503-443A-9D1F-61515DF8D4BF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{50E511A5-3157-4562-B28F-23CBA68899D9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="Casos de Testes" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Casos de Testes'!$A$1:$K$17</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Casos de Testes'!$A$1:$K$18</definedName>
   </definedNames>
   <calcPr calcId="191029" iterateDelta="1E-4"/>
   <extLst>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="156" uniqueCount="75">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="183" uniqueCount="81">
   <si>
     <t>ID</t>
   </si>
@@ -296,6 +296,30 @@
     <t>Não concluir cadastro de usuário
 Exibir mensagem "Formato inválido."</t>
   </si>
+  <si>
+    <t>CT-017</t>
+  </si>
+  <si>
+    <t>Exibe dados padrão do sistema, não há vinculo entre os dados cadastrados e os dados salvos. Há mais dados na tela de "Detalhes da conta" do que solicitados no cadastro</t>
+  </si>
+  <si>
+    <t>Concluir cadastro do usuário.
+ Exibir mensagem de boas vindas.
+Exibir nome e email cadastrados, exibir senha criptografada e demais campos vazios</t>
+  </si>
+  <si>
+    <t>1. Acessar página https://www.automationpratice.com.br/ 
+2. Clicar em Cadastro
+3.Inserir nome, email e senha
+4. Clicar no botão "Cadastro"
+5. Na Página Inicial, clicar em "Detalhes da conta"</t>
+  </si>
+  <si>
+    <t>Responsável</t>
+  </si>
+  <si>
+    <t>Bruna Lourenço</t>
+  </si>
 </sst>
 </file>
 
@@ -386,7 +410,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -460,6 +484,9 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -722,7 +749,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:N1001"/>
+  <dimension ref="A1:N999"/>
   <sheetFormatPr defaultColWidth="12.5703125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="10.85546875" customWidth="1"/>
@@ -735,6 +762,7 @@
     <col min="8" max="8" width="28.85546875" customWidth="1"/>
     <col min="9" max="9" width="36.140625" customWidth="1"/>
     <col min="10" max="11" width="12.85546875" customWidth="1"/>
+    <col min="12" max="12" width="17.140625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="15.75" x14ac:dyDescent="0.2">
@@ -771,7 +799,9 @@
       <c r="K1" s="12" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="2"/>
+      <c r="L1" s="12" t="s">
+        <v>79</v>
+      </c>
       <c r="M1" s="2"/>
       <c r="N1" s="2"/>
     </row>
@@ -804,13 +834,15 @@
         <v>18</v>
       </c>
       <c r="J2" s="17" t="str">
-        <f t="shared" ref="J2:J17" si="0">IF(H2=I2,"Passou","Falhou")</f>
+        <f t="shared" ref="J2:J18" si="0">IF(H2=I2,"Passou","Falhou")</f>
         <v>Passou</v>
       </c>
       <c r="K2" s="18">
         <v>46157</v>
       </c>
-      <c r="L2" s="6"/>
+      <c r="L2" s="26" t="s">
+        <v>80</v>
+      </c>
       <c r="M2" s="6"/>
       <c r="N2" s="6"/>
     </row>
@@ -849,7 +881,9 @@
       <c r="K3" s="18">
         <v>46157</v>
       </c>
-      <c r="L3" s="6"/>
+      <c r="L3" s="26" t="s">
+        <v>80</v>
+      </c>
       <c r="M3" s="6"/>
       <c r="N3" s="6"/>
     </row>
@@ -888,7 +922,9 @@
       <c r="K4" s="18">
         <v>46157</v>
       </c>
-      <c r="L4" s="6"/>
+      <c r="L4" s="26" t="s">
+        <v>80</v>
+      </c>
       <c r="M4" s="6"/>
       <c r="N4" s="6"/>
     </row>
@@ -927,7 +963,9 @@
       <c r="K5" s="18">
         <v>46157</v>
       </c>
-      <c r="L5" s="6"/>
+      <c r="L5" s="26" t="s">
+        <v>80</v>
+      </c>
       <c r="M5" s="6"/>
       <c r="N5" s="6"/>
     </row>
@@ -966,7 +1004,9 @@
       <c r="K6" s="18">
         <v>46157</v>
       </c>
-      <c r="L6" s="6"/>
+      <c r="L6" s="26" t="s">
+        <v>80</v>
+      </c>
       <c r="M6" s="6"/>
       <c r="N6" s="6"/>
     </row>
@@ -1005,7 +1045,9 @@
       <c r="K7" s="18">
         <v>46157</v>
       </c>
-      <c r="L7" s="6"/>
+      <c r="L7" s="26" t="s">
+        <v>80</v>
+      </c>
       <c r="M7" s="6"/>
       <c r="N7" s="6"/>
     </row>
@@ -1043,7 +1085,9 @@
       <c r="K8" s="24">
         <v>46157</v>
       </c>
-      <c r="L8" s="7"/>
+      <c r="L8" s="26" t="s">
+        <v>80</v>
+      </c>
       <c r="M8" s="7"/>
       <c r="N8" s="7"/>
     </row>
@@ -1082,7 +1126,9 @@
       <c r="K9" s="18">
         <v>46157</v>
       </c>
-      <c r="L9" s="6"/>
+      <c r="L9" s="26" t="s">
+        <v>80</v>
+      </c>
       <c r="M9" s="6"/>
       <c r="N9" s="6"/>
     </row>
@@ -1121,7 +1167,9 @@
       <c r="K10" s="18">
         <v>46157</v>
       </c>
-      <c r="L10" s="6"/>
+      <c r="L10" s="26" t="s">
+        <v>80</v>
+      </c>
       <c r="M10" s="6"/>
       <c r="N10" s="6"/>
     </row>
@@ -1160,7 +1208,9 @@
       <c r="K11" s="18">
         <v>46157</v>
       </c>
-      <c r="L11" s="6"/>
+      <c r="L11" s="26" t="s">
+        <v>80</v>
+      </c>
       <c r="M11" s="6"/>
       <c r="N11" s="6"/>
     </row>
@@ -1199,7 +1249,9 @@
       <c r="K12" s="18">
         <v>46157</v>
       </c>
-      <c r="L12" s="6"/>
+      <c r="L12" s="26" t="s">
+        <v>80</v>
+      </c>
       <c r="M12" s="6"/>
       <c r="N12" s="6"/>
     </row>
@@ -1238,7 +1290,9 @@
       <c r="K13" s="18">
         <v>46157</v>
       </c>
-      <c r="L13" s="6"/>
+      <c r="L13" s="26" t="s">
+        <v>80</v>
+      </c>
       <c r="M13" s="6"/>
       <c r="N13" s="6"/>
     </row>
@@ -1277,7 +1331,9 @@
       <c r="K14" s="18">
         <v>46157</v>
       </c>
-      <c r="L14" s="6"/>
+      <c r="L14" s="26" t="s">
+        <v>80</v>
+      </c>
       <c r="M14" s="6"/>
       <c r="N14" s="6"/>
     </row>
@@ -1316,7 +1372,9 @@
       <c r="K15" s="18">
         <v>46157</v>
       </c>
-      <c r="L15" s="6"/>
+      <c r="L15" s="26" t="s">
+        <v>80</v>
+      </c>
       <c r="M15" s="6"/>
       <c r="N15" s="6"/>
     </row>
@@ -1355,7 +1413,9 @@
       <c r="K16" s="18">
         <v>46157</v>
       </c>
-      <c r="L16" s="6"/>
+      <c r="L16" s="26" t="s">
+        <v>80</v>
+      </c>
       <c r="M16" s="6"/>
       <c r="N16" s="6"/>
     </row>
@@ -1394,24 +1454,52 @@
       <c r="K17" s="18">
         <v>46157</v>
       </c>
-      <c r="L17" s="6"/>
+      <c r="L17" s="26" t="s">
+        <v>80</v>
+      </c>
       <c r="M17" s="6"/>
       <c r="N17" s="6"/>
     </row>
-    <row r="18" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A18" s="3"/>
-      <c r="B18" s="4"/>
-      <c r="C18" s="5"/>
-      <c r="D18" s="3"/>
-      <c r="E18" s="5"/>
-      <c r="F18" s="4"/>
-      <c r="H18" s="4"/>
-      <c r="I18" s="4"/>
-      <c r="J18" s="3"/>
-      <c r="K18" s="6"/>
-      <c r="L18" s="6"/>
-      <c r="M18" s="6"/>
-      <c r="N18" s="6"/>
+    <row r="18" spans="1:14" s="8" customFormat="1" ht="120" x14ac:dyDescent="0.2">
+      <c r="A18" s="19" t="s">
+        <v>75</v>
+      </c>
+      <c r="B18" s="20" t="s">
+        <v>20</v>
+      </c>
+      <c r="C18" s="21" t="s">
+        <v>13</v>
+      </c>
+      <c r="D18" s="19" t="s">
+        <v>14</v>
+      </c>
+      <c r="E18" s="21" t="s">
+        <v>21</v>
+      </c>
+      <c r="F18" s="20" t="s">
+        <v>16</v>
+      </c>
+      <c r="G18" s="22" t="s">
+        <v>78</v>
+      </c>
+      <c r="H18" s="20" t="s">
+        <v>77</v>
+      </c>
+      <c r="I18" s="20" t="s">
+        <v>76</v>
+      </c>
+      <c r="J18" s="19" t="str">
+        <f t="shared" si="0"/>
+        <v>Falhou</v>
+      </c>
+      <c r="K18" s="24">
+        <v>46158</v>
+      </c>
+      <c r="L18" s="26" t="s">
+        <v>80</v>
+      </c>
+      <c r="M18" s="7"/>
+      <c r="N18" s="7"/>
     </row>
     <row r="19" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A19" s="3"/>
@@ -16128,38 +16216,8 @@
       <c r="M999" s="6"/>
       <c r="N999" s="6"/>
     </row>
-    <row r="1000" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A1000" s="3"/>
-      <c r="B1000" s="4"/>
-      <c r="C1000" s="5"/>
-      <c r="D1000" s="3"/>
-      <c r="E1000" s="5"/>
-      <c r="F1000" s="4"/>
-      <c r="H1000" s="4"/>
-      <c r="I1000" s="4"/>
-      <c r="J1000" s="3"/>
-      <c r="K1000" s="6"/>
-      <c r="L1000" s="6"/>
-      <c r="M1000" s="6"/>
-      <c r="N1000" s="6"/>
-    </row>
-    <row r="1001" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A1001" s="3"/>
-      <c r="B1001" s="4"/>
-      <c r="C1001" s="5"/>
-      <c r="D1001" s="3"/>
-      <c r="E1001" s="5"/>
-      <c r="F1001" s="4"/>
-      <c r="H1001" s="4"/>
-      <c r="I1001" s="4"/>
-      <c r="J1001" s="3"/>
-      <c r="K1001" s="6"/>
-      <c r="L1001" s="6"/>
-      <c r="M1001" s="6"/>
-      <c r="N1001" s="6"/>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:K17" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
+  <autoFilter ref="A1:K18" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
   <phoneticPr fontId="4" type="noConversion"/>
   <hyperlinks>
     <hyperlink ref="G2" r:id="rId1" display="https://www.automationpratice.com.br/" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
@@ -16178,8 +16236,9 @@
     <hyperlink ref="G16" r:id="rId14" display="https://www.automationpratice.com.br/" xr:uid="{00000000-0004-0000-0000-00000D000000}"/>
     <hyperlink ref="G17" r:id="rId15" display="https://www.automationpratice.com.br/" xr:uid="{00000000-0004-0000-0000-00000E000000}"/>
     <hyperlink ref="G8" r:id="rId16" display="https://www.automationpratice.com.br/" xr:uid="{E26F7D9E-1B7D-471D-98EE-490E75F7A9E8}"/>
+    <hyperlink ref="G18" r:id="rId17" display="https://www.automationpratice.com.br/" xr:uid="{24B2FC47-D6FF-4A3B-B03F-1A5617E3B575}"/>
   </hyperlinks>
   <pageMargins left="0.74791666666666701" right="0.74791666666666701" top="0.98402777777777795" bottom="0.98402777777777795" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId17"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId18"/>
 </worksheet>
 </file>
</xml_diff>